<commit_message>
Add updated Time_Profiling and shifted middleware to zs07 server
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Time_Profiling.xlsx
+++ b/Performance_Profiling/Time_Profiling.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26124"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5DD1BC3-C203-401A-8094-1455399DA1E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA4BAA05-81EF-4027-8004-C319DA36D42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="1.Profiling" sheetId="1" r:id="rId1"/>
+    <sheet name="2.Profiling" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="35">
   <si>
     <t>Time Unit: Seconds</t>
   </si>
@@ -36,6 +37,9 @@
     <t>Client instances: 1</t>
   </si>
   <si>
+    <t>Server: Local</t>
+  </si>
+  <si>
     <t>Functions</t>
   </si>
   <si>
@@ -118,6 +122,18 @@
   </si>
   <si>
     <t>Deviation (Error) Wall Time</t>
+  </si>
+  <si>
+    <t>Server: 10.0.2.87 (zs07)</t>
+  </si>
+  <si>
+    <t>1000 Key-Value Pairs</t>
+  </si>
+  <si>
+    <t>1000 Keys</t>
+  </si>
+  <si>
+    <t>Start:0, End:999</t>
   </si>
 </sst>
 </file>
@@ -144,7 +160,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -157,8 +173,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -203,25 +225,119 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -541,7 +657,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q80"/>
+  <dimension ref="A1:Q82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
@@ -552,7 +668,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="5" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
@@ -560,185 +676,180 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:17">
-      <c r="A3" s="11" t="s">
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="s">
+    </row>
+    <row r="4" spans="1:17">
+      <c r="A4" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="B4" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="C4" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="D4" s="23" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:17">
-      <c r="A4" s="5" t="s">
+      <c r="E4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="6">
+    </row>
+    <row r="5" spans="1:17">
+      <c r="A5" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="11">
         <v>5.1100005293846998E-7</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C5" s="12">
         <v>3.99641000058181E-4</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17">
-      <c r="A5" s="5" t="s">
+      <c r="D5" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="6">
+      <c r="E5" s="14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
+      <c r="A6" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4">
         <v>6.2999993133416801E-7</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C6" s="3">
         <v>1.13062979999085E-2</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="5" t="s">
+      <c r="D6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:17">
-      <c r="A6" s="5" t="s">
+      <c r="E6" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="6">
+    </row>
+    <row r="7" spans="1:17">
+      <c r="A7" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="4">
         <v>5.9300145949236996E-7</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C7" s="3">
         <v>2.3265749987331202E-3</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="5" t="s">
+      <c r="D7" t="s">
         <v>14</v>
       </c>
-      <c r="Q6" s="2"/>
-    </row>
-    <row r="7" spans="1:17">
-      <c r="A7" s="5" t="s">
+      <c r="E7" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="6">
+      <c r="Q7" s="2"/>
+    </row>
+    <row r="8" spans="1:17">
+      <c r="A8" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4">
         <v>9.5100040198303696E-7</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C8" s="24">
         <v>17.448833443999298</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="5" t="s">
+      <c r="D8" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
+      <c r="A9" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="4">
+        <v>5.7199940783903003E-7</v>
+      </c>
+      <c r="C9" s="3">
+        <v>7.8748550004092907E-3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
-      <c r="A8" s="5" t="s">
+    <row r="10" spans="1:17">
+      <c r="A10" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="4">
+        <v>7.9800156527198798E-7</v>
+      </c>
+      <c r="C10" s="24">
+        <v>17.2794635130012</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="6">
-        <v>5.7199940783903003E-7</v>
-      </c>
-      <c r="C8" s="7">
-        <v>7.8748550004092907E-3</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17">
-      <c r="A9" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="6">
-        <v>7.9800156527198798E-7</v>
-      </c>
-      <c r="C9" s="10">
-        <v>17.2794635130012</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17">
-      <c r="A10" s="5" t="s">
+    </row>
+    <row r="11" spans="1:17">
+      <c r="A11" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="4">
+        <v>7.4800118454732001E-7</v>
+      </c>
+      <c r="C11" s="24">
+        <v>17.235474565000899</v>
+      </c>
+      <c r="D11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17">
+      <c r="A12" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="4">
+        <v>9.5998984761536095E-8</v>
+      </c>
+      <c r="C12" s="3">
+        <v>9.7675260003597907E-3</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17">
+      <c r="A13" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="18">
+        <v>7.1999238571151998E-8</v>
+      </c>
+      <c r="C13" s="26">
+        <v>34.384241163999803</v>
+      </c>
+      <c r="D13" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="6">
-        <v>7.4800118454732001E-7</v>
-      </c>
-      <c r="C10" s="10">
-        <v>17.235474565000899</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17">
-      <c r="A11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="6">
-        <v>9.5998984761536095E-8</v>
-      </c>
-      <c r="C11" s="7">
-        <v>9.7675260003597907E-3</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17">
-      <c r="A12" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="6">
-        <v>7.1999238571151998E-8</v>
-      </c>
-      <c r="C12" s="10">
-        <v>34.384241163999803</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17">
-      <c r="B13" s="4"/>
-      <c r="C13" s="3"/>
+      <c r="E13" s="21" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="14" spans="1:17">
       <c r="B14" s="4"/>
@@ -753,79 +864,79 @@
       <c r="C16" s="3"/>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="5" t="s">
+      <c r="B17" s="4"/>
+      <c r="C17" s="3"/>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="11">
+        <v>5.9000012697651898E-7</v>
+      </c>
+      <c r="C18" s="12">
+        <v>0.179141746997629</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E18" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="4">
-        <v>5.9000012697651898E-7</v>
-      </c>
-      <c r="C17" s="3">
-        <v>0.179141746997629</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="4">
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="4">
         <v>6.4699997892603204E-7</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C19" s="3">
         <v>0.16894758000125801</v>
-      </c>
-      <c r="D18" t="s">
-        <v>26</v>
-      </c>
-      <c r="E18" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="4">
-        <v>5.4400152293965199E-7</v>
-      </c>
-      <c r="C19" s="3">
-        <v>0.17999452599906299</v>
       </c>
       <c r="D19" t="s">
         <v>27</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4">
+        <v>5.4400152293965199E-7</v>
+      </c>
+      <c r="C20" s="3">
+        <v>0.17999452599906299</v>
+      </c>
+      <c r="D20" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="17" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="4">
+      <c r="B21" s="18">
         <v>6.3800325733609498E-7</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C21" s="19">
         <v>0.35010583100302001</v>
       </c>
-      <c r="D20" t="s">
-        <v>26</v>
-      </c>
-      <c r="E20" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="B21" s="9"/>
-      <c r="C21" s="3"/>
+      <c r="D21" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="B22" s="4"/>
+      <c r="B22" s="5"/>
       <c r="C22" s="3"/>
     </row>
     <row r="23" spans="1:5">
@@ -836,105 +947,81 @@
       <c r="B24" s="4"/>
       <c r="C24" s="3"/>
     </row>
-    <row r="25" spans="1:5">
-      <c r="B25" s="4"/>
-      <c r="C25" s="3"/>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="B26" s="4"/>
-      <c r="C26" s="3"/>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="B27" s="4"/>
-      <c r="C27" s="3"/>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="B28" s="4"/>
-      <c r="C28" s="3"/>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="B29" s="4"/>
-      <c r="C29" s="3"/>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" t="s">
-        <v>28</v>
-      </c>
-      <c r="C30" s="4"/>
-    </row>
     <row r="31" spans="1:5">
-      <c r="A31" t="s">
+      <c r="B31" s="4"/>
+      <c r="C31" s="3"/>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="9">
+      <c r="C32" s="4"/>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" s="5">
         <v>2.08998244488611E-7</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
-      <c r="B32" s="4"/>
-      <c r="C32" s="3"/>
-    </row>
-    <row r="33" spans="2:3">
-      <c r="B33" s="4"/>
-      <c r="C33" s="3"/>
-    </row>
-    <row r="34" spans="2:3">
+    <row r="34" spans="1:3">
       <c r="B34" s="4"/>
       <c r="C34" s="3"/>
     </row>
-    <row r="35" spans="2:3">
+    <row r="35" spans="1:3">
       <c r="B35" s="4"/>
       <c r="C35" s="3"/>
     </row>
-    <row r="36" spans="2:3">
+    <row r="36" spans="1:3">
       <c r="B36" s="4"/>
       <c r="C36" s="3"/>
     </row>
-    <row r="37" spans="2:3">
+    <row r="37" spans="1:3">
       <c r="B37" s="4"/>
       <c r="C37" s="3"/>
     </row>
-    <row r="38" spans="2:3">
+    <row r="38" spans="1:3">
       <c r="B38" s="4"/>
       <c r="C38" s="3"/>
     </row>
-    <row r="39" spans="2:3">
+    <row r="39" spans="1:3">
       <c r="B39" s="4"/>
       <c r="C39" s="3"/>
     </row>
-    <row r="40" spans="2:3">
+    <row r="40" spans="1:3">
       <c r="B40" s="4"/>
       <c r="C40" s="3"/>
     </row>
-    <row r="41" spans="2:3">
+    <row r="41" spans="1:3">
       <c r="B41" s="4"/>
       <c r="C41" s="3"/>
     </row>
-    <row r="42" spans="2:3">
+    <row r="42" spans="1:3">
       <c r="B42" s="4"/>
       <c r="C42" s="3"/>
     </row>
-    <row r="43" spans="2:3">
+    <row r="43" spans="1:3">
       <c r="B43" s="4"/>
       <c r="C43" s="3"/>
     </row>
-    <row r="44" spans="2:3">
+    <row r="44" spans="1:3">
       <c r="B44" s="4"/>
       <c r="C44" s="3"/>
     </row>
-    <row r="45" spans="2:3">
+    <row r="45" spans="1:3">
       <c r="B45" s="4"/>
       <c r="C45" s="3"/>
     </row>
-    <row r="46" spans="2:3">
+    <row r="46" spans="1:3">
       <c r="B46" s="4"/>
       <c r="C46" s="3"/>
     </row>
-    <row r="47" spans="2:3">
+    <row r="47" spans="1:3">
       <c r="B47" s="4"/>
       <c r="C47" s="3"/>
     </row>
-    <row r="48" spans="2:3">
+    <row r="48" spans="1:3">
       <c r="B48" s="4"/>
       <c r="C48" s="3"/>
     </row>
@@ -1032,12 +1119,14 @@
     </row>
     <row r="72" spans="2:3">
       <c r="B72" s="4"/>
-      <c r="C72" s="1"/>
+      <c r="C72" s="3"/>
     </row>
     <row r="73" spans="2:3">
-      <c r="C73" s="1"/>
+      <c r="B73" s="4"/>
+      <c r="C73" s="3"/>
     </row>
     <row r="74" spans="2:3">
+      <c r="B74" s="4"/>
       <c r="C74" s="1"/>
     </row>
     <row r="75" spans="2:3">
@@ -1057,6 +1146,216 @@
     </row>
     <row r="80" spans="2:3">
       <c r="C80" s="1"/>
+    </row>
+    <row r="81" spans="3:3">
+      <c r="C81" s="1"/>
+    </row>
+    <row r="82" spans="3:3">
+      <c r="C82" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C82C9F3-A3C6-496B-9ECF-90CA2D4E4C55}">
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="36.140625" customWidth="1"/>
+    <col min="2" max="2" width="34.85546875" customWidth="1"/>
+    <col min="3" max="3" width="23.5703125" customWidth="1"/>
+    <col min="4" max="4" width="25.42578125" customWidth="1"/>
+    <col min="5" max="5" width="23" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="4">
+        <v>6.6699794842861497E-7</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.51838867100013797</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="4">
+        <v>6.4100095187313802E-7</v>
+      </c>
+      <c r="C6" s="3">
+        <v>0.427087743999436</v>
+      </c>
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="4">
+        <v>6.2799881561659202E-7</v>
+      </c>
+      <c r="C7" s="3">
+        <v>0.42318007900030302</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="18">
+        <v>7.6200012699700797E-7</v>
+      </c>
+      <c r="C8" s="19">
+        <v>0.59908431000076201</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="B9" s="4"/>
+      <c r="C9" s="3"/>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4">
+        <v>7.9999881563708101E-7</v>
+      </c>
+      <c r="C14" s="3">
+        <v>3.4945197119996001</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="4">
+        <v>6.1999890021979798E-7</v>
+      </c>
+      <c r="C15" s="3">
+        <v>3.0697713679983201</v>
+      </c>
+      <c r="D15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="4">
+        <v>8.4299972513690496E-7</v>
+      </c>
+      <c r="C16" s="3">
+        <v>3.4697741269992499</v>
+      </c>
+      <c r="D16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="18">
+        <v>8.0600148066878298E-7</v>
+      </c>
+      <c r="C17" s="19">
+        <v>5.7450908680002604</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update config replicas time profiling
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Time_Profiling.xlsx
+++ b/Performance_Profiling/Time_Profiling.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26124"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA4BAA05-81EF-4027-8004-C319DA36D42F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{166529A2-D05C-4265-B400-2F331236FAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.Profiling" sheetId="1" r:id="rId1"/>
     <sheet name="2.Profiling" sheetId="2" r:id="rId2"/>
+    <sheet name="3. Profiling" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="38">
   <si>
     <t>Time Unit: Seconds</t>
   </si>
@@ -40,6 +41,9 @@
     <t>Server: Local</t>
   </si>
   <si>
+    <t>Configs: NUM_REPLICAS = 10</t>
+  </si>
+  <si>
     <t>Functions</t>
   </si>
   <si>
@@ -134,6 +138,12 @@
   </si>
   <si>
     <t>Start:0, End:999</t>
+  </si>
+  <si>
+    <t>Client Instances: 1</t>
+  </si>
+  <si>
+    <t>Configs: NUM_REPLICAS = 30</t>
   </si>
 </sst>
 </file>
@@ -160,7 +170,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,6 +189,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -309,7 +325,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -338,6 +354,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -676,30 +694,33 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="28" t="s">
         <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" s="10" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" s="11">
         <v>5.1100005293846998E-7</v>
@@ -708,15 +729,15 @@
         <v>3.99641000058181E-4</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" s="15" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="4">
         <v>6.2999993133416801E-7</v>
@@ -725,15 +746,15 @@
         <v>1.13062979999085E-2</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B7" s="4">
         <v>5.9300145949236996E-7</v>
@@ -742,16 +763,16 @@
         <v>2.3265749987331202E-3</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q7" s="2"/>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" s="15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8" s="4">
         <v>9.5100040198303696E-7</v>
@@ -760,15 +781,15 @@
         <v>17.448833443999298</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" s="15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="4">
         <v>5.7199940783903003E-7</v>
@@ -777,15 +798,15 @@
         <v>7.8748550004092907E-3</v>
       </c>
       <c r="D9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" s="15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B10" s="4">
         <v>7.9800156527198798E-7</v>
@@ -794,15 +815,15 @@
         <v>17.2794635130012</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:17">
       <c r="A11" s="15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" s="4">
         <v>7.4800118454732001E-7</v>
@@ -811,15 +832,15 @@
         <v>17.235474565000899</v>
       </c>
       <c r="D11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" s="15" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="4">
         <v>9.5998984761536095E-8</v>
@@ -828,15 +849,15 @@
         <v>9.7675260003597907E-3</v>
       </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13" s="18">
         <v>7.1999238571151998E-8</v>
@@ -845,10 +866,10 @@
         <v>34.384241163999803</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -869,7 +890,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18" s="11">
         <v>5.9000012697651898E-7</v>
@@ -878,15 +899,15 @@
         <v>0.179141746997629</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B19" s="4">
         <v>6.4699997892603204E-7</v>
@@ -895,15 +916,15 @@
         <v>0.16894758000125801</v>
       </c>
       <c r="D19" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="16" t="s">
         <v>27</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B20" s="4">
         <v>5.4400152293965199E-7</v>
@@ -912,15 +933,15 @@
         <v>0.17999452599906299</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B21" s="18">
         <v>6.3800325733609498E-7</v>
@@ -929,10 +950,10 @@
         <v>0.35010583100302001</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -953,13 +974,13 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C32" s="4"/>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B33" s="5">
         <v>2.08998244488611E-7</v>
@@ -1165,7 +1186,7 @@
   <cols>
     <col min="1" max="1" width="36.140625" customWidth="1"/>
     <col min="2" max="2" width="34.85546875" customWidth="1"/>
-    <col min="3" max="3" width="23.5703125" customWidth="1"/>
+    <col min="3" max="3" width="28.85546875" customWidth="1"/>
     <col min="4" max="4" width="25.42578125" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
   </cols>
@@ -1180,29 +1201,32 @@
         <v>1</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="6" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B5" s="4">
         <v>6.6699794842861497E-7</v>
@@ -1211,15 +1235,15 @@
         <v>0.51838867100013797</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" s="4">
         <v>6.4100095187313802E-7</v>
@@ -1228,15 +1252,15 @@
         <v>0.427087743999436</v>
       </c>
       <c r="D6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="16" t="s">
         <v>33</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B7" s="4">
         <v>6.2799881561659202E-7</v>
@@ -1245,15 +1269,15 @@
         <v>0.42318007900030302</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B8" s="18">
         <v>7.6200012699700797E-7</v>
@@ -1262,10 +1286,10 @@
         <v>0.59908431000076201</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1274,24 +1298,24 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="6" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B14" s="4">
         <v>7.9999881563708101E-7</v>
@@ -1300,15 +1324,15 @@
         <v>3.4945197119996001</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="15" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B15" s="4">
         <v>6.1999890021979798E-7</v>
@@ -1317,15 +1341,15 @@
         <v>3.0697713679983201</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B16" s="4">
         <v>8.4299972513690496E-7</v>
@@ -1334,15 +1358,15 @@
         <v>3.4697741269992499</v>
       </c>
       <c r="D16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B17" s="18">
         <v>8.0600148066878298E-7</v>
@@ -1351,10 +1375,184 @@
         <v>5.7450908680002604</v>
       </c>
       <c r="D17" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3966AAAC-68E9-4693-8E19-B036A2F2FCF9}">
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="27.5703125" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" customWidth="1"/>
+    <col min="3" max="3" width="27.28515625" customWidth="1"/>
+    <col min="4" max="4" width="26.42578125" customWidth="1"/>
+    <col min="5" max="5" width="28.7109375" customWidth="1"/>
+    <col min="6" max="6" width="26.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="3">
+        <v>0.47043957799996799</v>
+      </c>
+      <c r="D5" s="22" t="s">
         <v>33</v>
       </c>
+      <c r="E5" s="16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="3"/>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="3"/>
+      <c r="D7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="18"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="3"/>
+      <c r="D15" t="s">
+        <v>22</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="3"/>
+      <c r="D16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="18"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="20" t="s">
+        <v>34</v>
+      </c>
       <c r="E17" s="21" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add documentation slides for design considerations
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Time_Profiling.xlsx
+++ b/Performance_Profiling/Time_Profiling.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26124"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25928"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{166529A2-D05C-4265-B400-2F331236FAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharding-ddms\Performance_Profiling\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B919AA3-BAB8-4FFB-B26B-6F6AE03C7EBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.Profiling" sheetId="1" r:id="rId1"/>
@@ -156,7 +161,7 @@
     <numFmt numFmtId="166" formatCode="0.00000000000000000000"/>
     <numFmt numFmtId="167" formatCode="0.000000000000000E+00"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -667,7 +672,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -676,7 +681,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q82"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
     <col min="2" max="2" width="30.5703125" customWidth="1"/>
@@ -685,12 +690,12 @@
     <col min="5" max="5" width="35.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -701,7 +706,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>4</v>
       </c>
@@ -718,7 +723,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>9</v>
       </c>
@@ -735,7 +740,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>11</v>
       </c>
@@ -752,7 +757,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>14</v>
       </c>
@@ -770,7 +775,7 @@
       </c>
       <c r="Q7" s="2"/>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
         <v>17</v>
       </c>
@@ -787,7 +792,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
         <v>19</v>
       </c>
@@ -804,7 +809,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
         <v>21</v>
       </c>
@@ -821,7 +826,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
         <v>23</v>
       </c>
@@ -838,7 +843,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
         <v>25</v>
       </c>
@@ -855,7 +860,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
         <v>26</v>
       </c>
@@ -872,23 +877,23 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B14" s="4"/>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B15" s="4"/>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B16" s="4"/>
       <c r="C16" s="3"/>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B17" s="4"/>
       <c r="C17" s="3"/>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
         <v>17</v>
       </c>
@@ -905,7 +910,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
         <v>21</v>
       </c>
@@ -922,7 +927,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
         <v>23</v>
       </c>
@@ -939,7 +944,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
         <v>26</v>
       </c>
@@ -956,29 +961,29 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B22" s="5"/>
       <c r="C22" s="3"/>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B23" s="4"/>
       <c r="C23" s="3"/>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B24" s="4"/>
       <c r="C24" s="3"/>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B31" s="4"/>
       <c r="C31" s="3"/>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>30</v>
       </c>
       <c r="C32" s="4"/>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -986,192 +991,192 @@
         <v>2.08998244488611E-7</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B34" s="4"/>
       <c r="C34" s="3"/>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B35" s="4"/>
       <c r="C35" s="3"/>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B36" s="4"/>
       <c r="C36" s="3"/>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B37" s="4"/>
       <c r="C37" s="3"/>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B38" s="4"/>
       <c r="C38" s="3"/>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B39" s="4"/>
       <c r="C39" s="3"/>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B40" s="4"/>
       <c r="C40" s="3"/>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B41" s="4"/>
       <c r="C41" s="3"/>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B42" s="4"/>
       <c r="C42" s="3"/>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B43" s="4"/>
       <c r="C43" s="3"/>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B44" s="4"/>
       <c r="C44" s="3"/>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B45" s="4"/>
       <c r="C45" s="3"/>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B46" s="4"/>
       <c r="C46" s="3"/>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B47" s="4"/>
       <c r="C47" s="3"/>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B48" s="4"/>
       <c r="C48" s="3"/>
     </row>
-    <row r="49" spans="2:3">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49" s="4"/>
       <c r="C49" s="3"/>
     </row>
-    <row r="50" spans="2:3">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50" s="4"/>
       <c r="C50" s="3"/>
     </row>
-    <row r="51" spans="2:3">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51" s="4"/>
       <c r="C51" s="3"/>
     </row>
-    <row r="52" spans="2:3">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52" s="4"/>
       <c r="C52" s="3"/>
     </row>
-    <row r="53" spans="2:3">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53" s="4"/>
       <c r="C53" s="3"/>
     </row>
-    <row r="54" spans="2:3">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54" s="4"/>
       <c r="C54" s="3"/>
     </row>
-    <row r="55" spans="2:3">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B55" s="4"/>
       <c r="C55" s="3"/>
     </row>
-    <row r="56" spans="2:3">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B56" s="4"/>
       <c r="C56" s="3"/>
     </row>
-    <row r="57" spans="2:3">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B57" s="4"/>
       <c r="C57" s="3"/>
     </row>
-    <row r="58" spans="2:3">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B58" s="4"/>
       <c r="C58" s="3"/>
     </row>
-    <row r="59" spans="2:3">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B59" s="4"/>
       <c r="C59" s="3"/>
     </row>
-    <row r="60" spans="2:3">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B60" s="4"/>
       <c r="C60" s="3"/>
     </row>
-    <row r="61" spans="2:3">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B61" s="4"/>
       <c r="C61" s="3"/>
     </row>
-    <row r="62" spans="2:3">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B62" s="4"/>
       <c r="C62" s="3"/>
     </row>
-    <row r="63" spans="2:3">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B63" s="4"/>
       <c r="C63" s="3"/>
     </row>
-    <row r="64" spans="2:3">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B64" s="4"/>
       <c r="C64" s="3"/>
     </row>
-    <row r="65" spans="2:3">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B65" s="4"/>
       <c r="C65" s="3"/>
     </row>
-    <row r="66" spans="2:3">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66" s="4"/>
       <c r="C66" s="3"/>
     </row>
-    <row r="67" spans="2:3">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67" s="4"/>
       <c r="C67" s="3"/>
     </row>
-    <row r="68" spans="2:3">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68" s="4"/>
       <c r="C68" s="3"/>
     </row>
-    <row r="69" spans="2:3">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B69" s="4"/>
       <c r="C69" s="3"/>
     </row>
-    <row r="70" spans="2:3">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70" s="4"/>
       <c r="C70" s="3"/>
     </row>
-    <row r="71" spans="2:3">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B71" s="4"/>
       <c r="C71" s="3"/>
     </row>
-    <row r="72" spans="2:3">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B72" s="4"/>
       <c r="C72" s="3"/>
     </row>
-    <row r="73" spans="2:3">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B73" s="4"/>
       <c r="C73" s="3"/>
     </row>
-    <row r="74" spans="2:3">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B74" s="4"/>
       <c r="C74" s="1"/>
     </row>
-    <row r="75" spans="2:3">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C75" s="1"/>
     </row>
-    <row r="76" spans="2:3">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C76" s="1"/>
     </row>
-    <row r="77" spans="2:3">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C77" s="1"/>
     </row>
-    <row r="78" spans="2:3">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C78" s="1"/>
     </row>
-    <row r="79" spans="2:3">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C79" s="1"/>
     </row>
-    <row r="80" spans="2:3">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C80" s="1"/>
     </row>
-    <row r="81" spans="3:3">
+    <row r="81" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C81" s="1"/>
     </row>
-    <row r="82" spans="3:3">
+    <row r="82" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C82" s="1"/>
     </row>
   </sheetData>
@@ -1182,7 +1187,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C82C9F3-A3C6-496B-9ECF-90CA2D4E4C55}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.140625" customWidth="1"/>
     <col min="2" max="2" width="34.85546875" customWidth="1"/>
@@ -1191,12 +1196,12 @@
     <col min="5" max="5" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1207,7 +1212,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
@@ -1224,7 +1229,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
         <v>17</v>
       </c>
@@ -1241,7 +1246,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>21</v>
       </c>
@@ -1258,7 +1263,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>23</v>
       </c>
@@ -1275,7 +1280,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
         <v>26</v>
       </c>
@@ -1292,11 +1297,11 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B9" s="4"/>
       <c r="C9" s="3"/>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>4</v>
       </c>
@@ -1313,7 +1318,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
         <v>17</v>
       </c>
@@ -1330,7 +1335,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
         <v>21</v>
       </c>
@@ -1347,7 +1352,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
         <v>23</v>
       </c>
@@ -1364,7 +1369,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
         <v>26</v>
       </c>
@@ -1389,7 +1394,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3966AAAC-68E9-4693-8E19-B036A2F2FCF9}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" customWidth="1"/>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
@@ -1399,12 +1404,12 @@
     <col min="6" max="6" width="26.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="29" t="s">
         <v>36</v>
       </c>
@@ -1415,7 +1420,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
@@ -1432,7 +1437,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
         <v>17</v>
       </c>
@@ -1447,7 +1452,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>21</v>
       </c>
@@ -1460,7 +1465,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
         <v>23</v>
       </c>
@@ -1473,7 +1478,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
         <v>26</v>
       </c>
@@ -1486,7 +1491,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>4</v>
       </c>
@@ -1503,7 +1508,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
         <v>17</v>
       </c>
@@ -1516,7 +1521,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
         <v>21</v>
       </c>
@@ -1529,7 +1534,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
         <v>23</v>
       </c>
@@ -1542,7 +1547,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
Add optimized hash function and config parameters
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Time_Profiling.xlsx
+++ b/Performance_Profiling/Time_Profiling.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharding-ddms\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B919AA3-BAB8-4FFB-B26B-6F6AE03C7EBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{376F07B7-C99C-4903-8C61-6688735A76BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1.Profiling" sheetId="1" r:id="rId1"/>
@@ -46,9 +46,6 @@
     <t>Server: Local</t>
   </si>
   <si>
-    <t>Configs: NUM_REPLICAS = 10</t>
-  </si>
-  <si>
     <t>Functions</t>
   </si>
   <si>
@@ -148,7 +145,10 @@
     <t>Client Instances: 1</t>
   </si>
   <si>
-    <t>Configs: NUM_REPLICAS = 30</t>
+    <t>Configs: VIRTUAL_SITES = 5</t>
+  </si>
+  <si>
+    <t>Configs: VIRTUAL_SITES = 10</t>
   </si>
 </sst>
 </file>
@@ -703,29 +703,29 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="C4" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="E4" s="14" t="s">
         <v>7</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="11">
         <v>5.1100005293846998E-7</v>
@@ -734,15 +734,15 @@
         <v>3.99641000058181E-4</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="4">
         <v>6.2999993133416801E-7</v>
@@ -751,15 +751,15 @@
         <v>1.13062979999085E-2</v>
       </c>
       <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="16" t="s">
         <v>12</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" s="4">
         <v>5.9300145949236996E-7</v>
@@ -768,16 +768,16 @@
         <v>2.3265749987331202E-3</v>
       </c>
       <c r="D7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="16" t="s">
         <v>15</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>16</v>
       </c>
       <c r="Q7" s="2"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" s="4">
         <v>9.5100040198303696E-7</v>
@@ -786,15 +786,15 @@
         <v>17.448833443999298</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="4">
         <v>5.7199940783903003E-7</v>
@@ -803,15 +803,15 @@
         <v>7.8748550004092907E-3</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" s="4">
         <v>7.9800156527198798E-7</v>
@@ -820,15 +820,15 @@
         <v>17.2794635130012</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E10" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" s="4">
         <v>7.4800118454732001E-7</v>
@@ -837,15 +837,15 @@
         <v>17.235474565000899</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" s="4">
         <v>9.5998984761536095E-8</v>
@@ -854,15 +854,15 @@
         <v>9.7675260003597907E-3</v>
       </c>
       <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="16" t="s">
         <v>15</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13" s="18">
         <v>7.1999238571151998E-8</v>
@@ -871,10 +871,10 @@
         <v>34.384241163999803</v>
       </c>
       <c r="D13" s="27" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
@@ -895,7 +895,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" s="11">
         <v>5.9000012697651898E-7</v>
@@ -904,15 +904,15 @@
         <v>0.179141746997629</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19" s="4">
         <v>6.4699997892603204E-7</v>
@@ -921,15 +921,15 @@
         <v>0.16894758000125801</v>
       </c>
       <c r="D19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B20" s="4">
         <v>5.4400152293965199E-7</v>
@@ -938,15 +938,15 @@
         <v>0.17999452599906299</v>
       </c>
       <c r="D20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" s="18">
         <v>6.3800325733609498E-7</v>
@@ -955,10 +955,10 @@
         <v>0.35010583100302001</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -979,13 +979,13 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C32" s="4"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B33" s="5">
         <v>2.08998244488611E-7</v>
@@ -1206,32 +1206,32 @@
         <v>1</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>7</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="4">
         <v>6.6699794842861497E-7</v>
@@ -1240,15 +1240,15 @@
         <v>0.51838867100013797</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" s="4">
         <v>6.4100095187313802E-7</v>
@@ -1257,15 +1257,15 @@
         <v>0.427087743999436</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" s="4">
         <v>6.2799881561659202E-7</v>
@@ -1274,15 +1274,15 @@
         <v>0.42318007900030302</v>
       </c>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8" s="18">
         <v>7.6200012699700797E-7</v>
@@ -1291,10 +1291,10 @@
         <v>0.59908431000076201</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1303,24 +1303,24 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="C13" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="E13" s="8" t="s">
         <v>7</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" s="4">
         <v>7.9999881563708101E-7</v>
@@ -1329,15 +1329,15 @@
         <v>3.4945197119996001</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="4">
         <v>6.1999890021979798E-7</v>
@@ -1346,15 +1346,15 @@
         <v>3.0697713679983201</v>
       </c>
       <c r="D15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" s="4">
         <v>8.4299972513690496E-7</v>
@@ -1363,15 +1363,15 @@
         <v>3.4697741269992499</v>
       </c>
       <c r="D16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17" s="18">
         <v>8.0600148066878298E-7</v>
@@ -1380,10 +1380,10 @@
         <v>5.7450908680002604</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1411,153 +1411,153 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="28" t="s">
         <v>36</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="28" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>7</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="3">
         <v>0.47043957799996799</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="3"/>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="3"/>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8" s="18"/>
       <c r="C8" s="19"/>
       <c r="D8" s="20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E8" s="21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="C13" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="E13" s="8" t="s">
         <v>7</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="3"/>
       <c r="D14" s="22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="3"/>
       <c r="D15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="3"/>
       <c r="D16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17" s="18"/>
       <c r="C17" s="19"/>
       <c r="D17" s="20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>